<commit_message>
Fixup comments in example excel files fmudesign
</commit_message>
<xml_diff>
--- a/src/fmudesign/examples/fmudesign_ex_montecarlo.xlsx
+++ b/src/fmudesign/examples/fmudesign_ex_montecarlo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/LEVJE/dev_komodo/semeio/src/semeio/fmudesign/examples/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/LEVJE/project/ert/src/fmudesign/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09AF5827-27A7-2F47-91FE-98C0E2F04E49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1670C82C-859D-B64D-8765-0A1C1837F77B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="27180" windowHeight="18420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="20520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="general_input" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t>Specifies that this is a setup for a onebyone design</t>
+          <t>Specifies that this is a setup for a onebyone design.</t>
         </r>
       </text>
     </comment>
@@ -57,7 +57,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t xml:space="preserve">Number of repeated rms_seeds per sensitivity/sensitivity case. 
+          <t xml:space="preserve">Number of repeated rms_seeds per sensitivity/sensitivity case.
 </t>
         </r>
         <r>
@@ -68,7 +68,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t>This is overridden if the number of realisations is specified in the “numreal” column in designinput.</t>
+          <t>This is overridden if the number of realisations is specified in the "numreal" column in designinput.</t>
         </r>
       </text>
     </comment>
@@ -93,7 +93,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t xml:space="preserve">- default gives seed numbers 1000, 1001, 1002, ...
+          <t xml:space="preserve">- default: Use seed numbers 1000, 1001, 1002, ...
 </t>
         </r>
         <r>
@@ -104,7 +104,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t xml:space="preserve">- None (seed number is not added as parameter in output spreadsheet) 
+          <t xml:space="preserve">- None: Seed number is not added as parameter in output spreadsheet.
 </t>
         </r>
         <r>
@@ -115,7 +115,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t>- filename for file with list of seeds in ert/input/distributions/</t>
+          <t>- Name of file with seeds in the first column (.xlsx, .csv or .txt). The path can be absolute or relative (to input file).</t>
         </r>
       </text>
     </comment>
@@ -140,7 +140,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t xml:space="preserve">- None
+          <t xml:space="preserve">- None.
 </t>
         </r>
         <r>
@@ -151,7 +151,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t xml:space="preserve">- name of sheet in this workbook with background parameters
+          <t xml:space="preserve">- Name of sheet in this workbook with background parameters.
 </t>
         </r>
         <r>
@@ -162,7 +162,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t>- Name of external file with background parameters. Must end with .xlsx or .csv and be readable as pandas dataframe with parameter names as column headers. The path can be absolute, or relative (to the location of this file)</t>
+          <t>- Name of external file with background parameters. Must end with .xlsx or .csv and be readable as pandas dataframe with parameter names as column headers. The path can be absolute or relative (to the location of this file).</t>
         </r>
       </text>
     </comment>
@@ -176,7 +176,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t xml:space="preserve">Seed user for random number generator (RNG). Alternatives:
+          <t xml:space="preserve">Seed used for random number generator (RNG). Alternatives:
 </t>
         </r>
         <r>
@@ -187,7 +187,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t xml:space="preserve"> - A number (e.g. a six digit number like 294284) to see the RNG.
+          <t xml:space="preserve">- A number (e.g. a six-digit number like 294284) to seed the RNG.
 </t>
         </r>
         <r>
@@ -198,7 +198,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t xml:space="preserve"> - None. The RNG will not be seeded and analysis will not be reproducible.</t>
+          <t>- None: The RNG will not be seeded and analysis will not be reproducible.</t>
         </r>
       </text>
     </comment>
@@ -223,7 +223,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t xml:space="preserve">- If ‘correlation_iterations’ is set to 0, then only Iman-Conover is used.
+          <t xml:space="preserve">- If "correlation_iterations" is set to 0, then only Iman-Conover is used.
 </t>
         </r>
         <r>
@@ -234,7 +234,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t>- If ‘correlation_iterations’ is a positive integer, then random swaps will be performed to improve the correlation. This takes a bit longer, but typically leads to observec orrelation that is closer to desired correlation, especially when variables are far from Gaussian (normal distribution). A value of 999 is a good starting point.</t>
+          <t>- If "correlation_iterations" is a positive integer, then random swaps will be performed to improve the correlation. This takes a bit longer, but typically leads to observed correlation that is closer to desired correlation, especially when variables are far from Gaussian (normal distribution). A value of 999 is a good starting point.</t>
         </r>
       </text>
     </comment>
@@ -257,7 +257,7 @@
             <rFont val="Calibri"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve"> -  joint  (default): Adding, removing, or reordering parameters may change samples for other parameters.
+          <t xml:space="preserve">- joint (default): Adding, removing, or reordering parameters may change samples for other parameters.
 </t>
         </r>
         <r>
@@ -267,7 +267,7 @@
             <rFont val="Calibri"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">  -  independent : Samples for unchanged parameters and correlation groups stay the same, provided neither distribution_seed nor the sample size changes. </t>
+          <t>- independent: Samples for unchanged parameters and correlation groups stay the same, provided neither distribution_seed nor the sample size changes.</t>
         </r>
       </text>
     </comment>
@@ -291,7 +291,7 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t xml:space="preserve">These are the distributions available.
+          <t xml:space="preserve">These are the distributions available:
 </t>
         </r>
         <r>

</xml_diff>